<commit_message>
corregido endpoint para traer todas las UC de un usuario
</commit_message>
<xml_diff>
--- a/BACKEND/EjemplosExcels/file-AF.xlsx
+++ b/BACKEND/EjemplosExcels/file-AF.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\SVS-System\BACKEND\EjemplosExcels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F550E0-362F-49DA-B60B-842EF3ED287B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D46DE0A7-6025-4E25-824E-87FADEAD095B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -678,7 +678,7 @@
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="11">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -711,7 +711,7 @@
       </c>
       <c r="J3" s="10"/>
       <c r="K3" s="11">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -744,7 +744,7 @@
       </c>
       <c r="J4" s="10"/>
       <c r="K4" s="11">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -779,7 +779,7 @@
         <v>33</v>
       </c>
       <c r="K5" s="11">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -814,7 +814,7 @@
         <v>33</v>
       </c>
       <c r="K6" s="11">
-        <v>99</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -847,7 +847,7 @@
       </c>
       <c r="J7" s="10"/>
       <c r="K7" s="11">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
modificado service de unidad curricular para ampliar la respuesta al buscar 1 o mas UCs
</commit_message>
<xml_diff>
--- a/BACKEND/EjemplosExcels/file-AF.xlsx
+++ b/BACKEND/EjemplosExcels/file-AF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\SVS-System\BACKEND\EjemplosExcels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D46DE0A7-6025-4E25-824E-87FADEAD095B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE425A1-A60D-4F95-95FA-40A13263A53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="50">
   <si>
     <t>Apellido y nombre</t>
   </si>
@@ -173,6 +173,9 @@
   </si>
   <si>
     <t>DNI - 49062828</t>
+  </si>
+  <si>
+    <t>1ro</t>
   </si>
 </sst>
 </file>
@@ -677,8 +680,8 @@
         <v>16</v>
       </c>
       <c r="J2" s="10"/>
-      <c r="K2" s="11">
-        <v>33</v>
+      <c r="K2" s="11" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -710,8 +713,8 @@
         <v>16</v>
       </c>
       <c r="J3" s="10"/>
-      <c r="K3" s="11">
-        <v>33</v>
+      <c r="K3" s="11" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -743,8 +746,8 @@
         <v>28</v>
       </c>
       <c r="J4" s="10"/>
-      <c r="K4" s="11">
-        <v>33</v>
+      <c r="K4" s="11" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -778,8 +781,8 @@
       <c r="J5" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="K5" s="11">
-        <v>33</v>
+      <c r="K5" s="11" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -813,8 +816,8 @@
       <c r="J6" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="K6" s="11">
-        <v>33</v>
+      <c r="K6" s="11" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -846,8 +849,8 @@
         <v>16</v>
       </c>
       <c r="J7" s="10"/>
-      <c r="K7" s="11">
-        <v>33</v>
+      <c r="K7" s="11" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Traido Backend desde feature/service-material_clase-taiel
</commit_message>
<xml_diff>
--- a/BACKEND/EjemplosExcels/file-AF.xlsx
+++ b/BACKEND/EjemplosExcels/file-AF.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\SVS-System\BACKEND\EjemplosExcels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D46DE0A7-6025-4E25-824E-87FADEAD095B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F550E0-362F-49DA-B60B-842EF3ED287B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -678,7 +678,7 @@
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="11">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -711,7 +711,7 @@
       </c>
       <c r="J3" s="10"/>
       <c r="K3" s="11">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -744,7 +744,7 @@
       </c>
       <c r="J4" s="10"/>
       <c r="K4" s="11">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -779,7 +779,7 @@
         <v>33</v>
       </c>
       <c r="K5" s="11">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -814,7 +814,7 @@
         <v>33</v>
       </c>
       <c r="K6" s="11">
-        <v>33</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -847,7 +847,7 @@
       </c>
       <c r="J7" s="10"/>
       <c r="K7" s="11">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>